<commit_message>
added auto update of graphs to my website
</commit_message>
<xml_diff>
--- a/data/gas_prices.xlsx
+++ b/data/gas_prices.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I641"/>
+  <dimension ref="A1:I701"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25392,10 +25392,8 @@
       </c>
     </row>
     <row r="622">
-      <c r="A622" t="inlineStr">
-        <is>
-          <t>65515</t>
-        </is>
+      <c r="A622" t="n">
+        <v>65515</v>
       </c>
       <c r="B622" t="inlineStr">
         <is>
@@ -25435,10 +25433,8 @@
       </c>
     </row>
     <row r="623">
-      <c r="A623" t="inlineStr">
-        <is>
-          <t>77205</t>
-        </is>
+      <c r="A623" t="n">
+        <v>77205</v>
       </c>
       <c r="B623" t="inlineStr">
         <is>
@@ -25478,10 +25474,8 @@
       </c>
     </row>
     <row r="624">
-      <c r="A624" t="inlineStr">
-        <is>
-          <t>77223</t>
-        </is>
+      <c r="A624" t="n">
+        <v>77223</v>
       </c>
       <c r="B624" t="inlineStr">
         <is>
@@ -25509,10 +25503,8 @@
       <c r="I624" t="inlineStr"/>
     </row>
     <row r="625">
-      <c r="A625" t="inlineStr">
-        <is>
-          <t>65514</t>
-        </is>
+      <c r="A625" t="n">
+        <v>65514</v>
       </c>
       <c r="B625" t="inlineStr">
         <is>
@@ -25552,10 +25544,8 @@
       </c>
     </row>
     <row r="626">
-      <c r="A626" t="inlineStr">
-        <is>
-          <t>77232</t>
-        </is>
+      <c r="A626" t="n">
+        <v>77232</v>
       </c>
       <c r="B626" t="inlineStr">
         <is>
@@ -25595,10 +25585,8 @@
       </c>
     </row>
     <row r="627">
-      <c r="A627" t="inlineStr">
-        <is>
-          <t>77202</t>
-        </is>
+      <c r="A627" t="n">
+        <v>77202</v>
       </c>
       <c r="B627" t="inlineStr">
         <is>
@@ -25638,10 +25626,8 @@
       </c>
     </row>
     <row r="628">
-      <c r="A628" t="inlineStr">
-        <is>
-          <t>86650</t>
-        </is>
+      <c r="A628" t="n">
+        <v>86650</v>
       </c>
       <c r="B628" t="inlineStr">
         <is>
@@ -25681,10 +25667,8 @@
       </c>
     </row>
     <row r="629">
-      <c r="A629" t="inlineStr">
-        <is>
-          <t>77218</t>
-        </is>
+      <c r="A629" t="n">
+        <v>77218</v>
       </c>
       <c r="B629" t="inlineStr">
         <is>
@@ -25724,10 +25708,8 @@
       </c>
     </row>
     <row r="630">
-      <c r="A630" t="inlineStr">
-        <is>
-          <t>77243</t>
-        </is>
+      <c r="A630" t="n">
+        <v>77243</v>
       </c>
       <c r="B630" t="inlineStr">
         <is>
@@ -25767,10 +25749,8 @@
       </c>
     </row>
     <row r="631">
-      <c r="A631" t="inlineStr">
-        <is>
-          <t>77235</t>
-        </is>
+      <c r="A631" t="n">
+        <v>77235</v>
       </c>
       <c r="B631" t="inlineStr">
         <is>
@@ -25810,10 +25790,8 @@
       </c>
     </row>
     <row r="632">
-      <c r="A632" t="inlineStr">
-        <is>
-          <t>77228</t>
-        </is>
+      <c r="A632" t="n">
+        <v>77228</v>
       </c>
       <c r="B632" t="inlineStr">
         <is>
@@ -25853,10 +25831,8 @@
       </c>
     </row>
     <row r="633">
-      <c r="A633" t="inlineStr">
-        <is>
-          <t>69163</t>
-        </is>
+      <c r="A633" t="n">
+        <v>69163</v>
       </c>
       <c r="B633" t="inlineStr">
         <is>
@@ -25896,10 +25872,8 @@
       </c>
     </row>
     <row r="634">
-      <c r="A634" t="inlineStr">
-        <is>
-          <t>109205</t>
-        </is>
+      <c r="A634" t="n">
+        <v>109205</v>
       </c>
       <c r="B634" t="inlineStr">
         <is>
@@ -25939,10 +25913,8 @@
       </c>
     </row>
     <row r="635">
-      <c r="A635" t="inlineStr">
-        <is>
-          <t>65512</t>
-        </is>
+      <c r="A635" t="n">
+        <v>65512</v>
       </c>
       <c r="B635" t="inlineStr">
         <is>
@@ -25982,10 +25954,8 @@
       </c>
     </row>
     <row r="636">
-      <c r="A636" t="inlineStr">
-        <is>
-          <t>83384</t>
-        </is>
+      <c r="A636" t="n">
+        <v>83384</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
@@ -26025,10 +25995,8 @@
       </c>
     </row>
     <row r="637">
-      <c r="A637" t="inlineStr">
-        <is>
-          <t>77015</t>
-        </is>
+      <c r="A637" t="n">
+        <v>77015</v>
       </c>
       <c r="B637" t="inlineStr">
         <is>
@@ -26068,10 +26036,8 @@
       </c>
     </row>
     <row r="638">
-      <c r="A638" t="inlineStr">
-        <is>
-          <t>107728</t>
-        </is>
+      <c r="A638" t="n">
+        <v>107728</v>
       </c>
       <c r="B638" t="inlineStr">
         <is>
@@ -26111,10 +26077,8 @@
       </c>
     </row>
     <row r="639">
-      <c r="A639" t="inlineStr">
-        <is>
-          <t>65572</t>
-        </is>
+      <c r="A639" t="n">
+        <v>65572</v>
       </c>
       <c r="B639" t="inlineStr">
         <is>
@@ -26154,10 +26118,8 @@
       </c>
     </row>
     <row r="640">
-      <c r="A640" t="inlineStr">
-        <is>
-          <t>65511</t>
-        </is>
+      <c r="A640" t="n">
+        <v>65511</v>
       </c>
       <c r="B640" t="inlineStr">
         <is>
@@ -26197,10 +26159,8 @@
       </c>
     </row>
     <row r="641">
-      <c r="A641" t="inlineStr">
-        <is>
-          <t>65556</t>
-        </is>
+      <c r="A641" t="n">
+        <v>65556</v>
       </c>
       <c r="B641" t="inlineStr">
         <is>
@@ -26237,6 +26197,2374 @@
       </c>
       <c r="I641" t="n">
         <v>184.9</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="n">
+        <v>65542</v>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>3250 MacDonald St</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.2573819, 'Longitude': -123.1680407}</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>2025-08-20T01:45:00.108Z</t>
+        </is>
+      </c>
+      <c r="G642" t="n">
+        <v>162.9</v>
+      </c>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>2025-08-18T20:00:38.663Z</t>
+        </is>
+      </c>
+      <c r="I642" t="n">
+        <v>191.9</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="n">
+        <v>65533</v>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>4615 Arbutus St</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.2449719, 'Longitude': -123.1540385}</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>2025-08-20T02:41:12.206Z</t>
+        </is>
+      </c>
+      <c r="G643" t="n">
+        <v>162.9</v>
+      </c>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>2025-08-18T20:01:38.582Z</t>
+        </is>
+      </c>
+      <c r="I643" t="n">
+        <v>191.9</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="n">
+        <v>83068</v>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Esso</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>3205 Arbutus St</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.256927568207, 'Longitude': -123.153288960457}</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr"/>
+      <c r="G644" t="inlineStr"/>
+      <c r="H644" t="inlineStr"/>
+      <c r="I644" t="inlineStr"/>
+    </row>
+    <row r="645">
+      <c r="A645" t="n">
+        <v>65562</v>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>2808 W Broadway</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.263883932125, 'Longitude': -123.168604373932}</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>2025-08-20T00:17:36.374Z</t>
+        </is>
+      </c>
+      <c r="G645" t="n">
+        <v>163.9</v>
+      </c>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>2025-08-20T00:17:36.405Z</t>
+        </is>
+      </c>
+      <c r="I645" t="n">
+        <v>188.9</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="n">
+        <v>113305</v>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>3596 W 41st Ave</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.234385296079, 'Longitude': -123.184762001038}</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>2025-08-20T02:29:29.571Z</t>
+        </is>
+      </c>
+      <c r="G646" t="n">
+        <v>163.9</v>
+      </c>
+      <c r="H646" t="inlineStr"/>
+      <c r="I646" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="n">
+        <v>65570</v>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>2103 W Broadway</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.264135981257, 'Longitude': -123.153326511383}</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:35:04.188Z</t>
+        </is>
+      </c>
+      <c r="G647" t="n">
+        <v>162.9</v>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>2025-08-19T17:50:59.425Z</t>
+        </is>
+      </c>
+      <c r="I647" t="n">
+        <v>197.9</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="n">
+        <v>65554</v>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Esso</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>1795 W Broadway</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.264037962303, 'Longitude': -123.145408630371}</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:33:38.071Z</t>
+        </is>
+      </c>
+      <c r="G648" t="n">
+        <v>162.9</v>
+      </c>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:44:20.091Z</t>
+        </is>
+      </c>
+      <c r="I648" t="n">
+        <v>189.9</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="n">
+        <v>65571</v>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>4314 W 10th Ave</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.263533861752, 'Longitude': -123.203430175781}</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>2025-08-19T21:12:07.564Z</t>
+        </is>
+      </c>
+      <c r="G649" t="n">
+        <v>167.9</v>
+      </c>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>2025-08-19T16:29:09.259Z</t>
+        </is>
+      </c>
+      <c r="I649" t="n">
+        <v>197.9</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="n">
+        <v>65565</v>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>1896 W 4th Ave</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.267881559667, 'Longitude': -123.14772605896}</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>2025-08-20T02:51:14.843Z</t>
+        </is>
+      </c>
+      <c r="G650" t="n">
+        <v>158.9</v>
+      </c>
+      <c r="H650" t="inlineStr"/>
+      <c r="I650" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="n">
+        <v>32376</v>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>1503 W 41st Ave</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.234634576953, 'Longitude': -123.139971792698}</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>2025-08-20T01:47:31.224Z</t>
+        </is>
+      </c>
+      <c r="G651" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>2025-08-19T22:30:08.915Z</t>
+        </is>
+      </c>
+      <c r="I651" t="n">
+        <v>189.9</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="n">
+        <v>65549</v>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Esso</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>5702 Granville St</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.234036184118, 'Longitude': -123.139244914055}</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>2025-08-20T01:29:49.623Z</t>
+        </is>
+      </c>
+      <c r="G652" t="n">
+        <v>157.9</v>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>2025-08-19T19:13:29.302Z</t>
+        </is>
+      </c>
+      <c r="I652" t="n">
+        <v>196.9</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="n">
+        <v>65543</v>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>1900 Burrard St</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.2685375, 'Longitude': -123.1453067}</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>2025-08-20T02:51:31.870Z</t>
+        </is>
+      </c>
+      <c r="G653" t="n">
+        <v>164.9</v>
+      </c>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>2025-08-19T22:57:09.641Z</t>
+        </is>
+      </c>
+      <c r="I653" t="n">
+        <v>191.9</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="n">
+        <v>65563</v>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>1743 Burrard St</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.270429790667, 'Longitude': -123.145886063576}</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>2025-08-20T02:51:19.264Z</t>
+        </is>
+      </c>
+      <c r="G654" t="n">
+        <v>158.9</v>
+      </c>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>2025-08-20T01:53:03.891Z</t>
+        </is>
+      </c>
+      <c r="I654" t="n">
+        <v>184.9</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="n">
+        <v>72747</v>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Esso</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>1010 W King Edward Ave</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.249188, 'Longitude': -123.127767}</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:43:58.820Z</t>
+        </is>
+      </c>
+      <c r="G655" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:43:58.867Z</t>
+        </is>
+      </c>
+      <c r="I655" t="n">
+        <v>185.9</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="n">
+        <v>32375</v>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>4110 Oak St</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.24894071957, 'Longitude': -123.127040863037}</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:16:00.265Z</t>
+        </is>
+      </c>
+      <c r="G656" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>2025-08-19T19:13:19.073Z</t>
+        </is>
+      </c>
+      <c r="I656" t="n">
+        <v>191.9</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="n">
+        <v>65564</v>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>5680 Oak St</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.234217162181, 'Longitude': -123.127684593201}</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:14:02.226Z</t>
+        </is>
+      </c>
+      <c r="G657" t="n">
+        <v>157.9</v>
+      </c>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>2025-08-19T19:12:49.425Z</t>
+        </is>
+      </c>
+      <c r="I657" t="n">
+        <v>189.9</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="n">
+        <v>32372</v>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Esso</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>6525 Oak St</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.226226639452, 'Longitude': -123.128687739372}</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:15:00.452Z</t>
+        </is>
+      </c>
+      <c r="G658" t="n">
+        <v>157.9</v>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>2025-08-19T19:29:56.703Z</t>
+        </is>
+      </c>
+      <c r="I658" t="n">
+        <v>197.9</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="n">
+        <v>9707</v>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Esso</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>1205 Burrard St</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.279145231489, 'Longitude': -123.12982365489}</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:44:10.433Z</t>
+        </is>
+      </c>
+      <c r="G659" t="n">
+        <v>160.9</v>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:44:10.464Z</t>
+        </is>
+      </c>
+      <c r="I659" t="n">
+        <v>195.9</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="n">
+        <v>65566</v>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>8072 Granville St</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.212495055855, 'Longitude': -123.14013004303}</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>2025-08-20T02:28:24.653Z</t>
+        </is>
+      </c>
+      <c r="G660" t="n">
+        <v>165.9</v>
+      </c>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>2025-08-19T19:30:08.359Z</t>
+        </is>
+      </c>
+      <c r="I660" t="n">
+        <v>197.9</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="n">
+        <v>65572</v>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>8686 Granville St</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.207280329467, 'Longitude': -123.140280246735}</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:38:53</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>2025-08-20T01:07:36.107Z</t>
+        </is>
+      </c>
+      <c r="G661" t="n">
+        <v>167.9</v>
+      </c>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>2025-08-19T19:31:11.263Z</t>
+        </is>
+      </c>
+      <c r="I661" t="n">
+        <v>197.9</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="n">
+        <v>65558</v>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>1390 E 33rd Ave</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.240045470021, 'Longitude': -123.076765537262}</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:29:52.466Z</t>
+        </is>
+      </c>
+      <c r="G662" t="n">
+        <v>153.9</v>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:21:41.203Z</t>
+        </is>
+      </c>
+      <c r="I662" t="n">
+        <v>177.9</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="n">
+        <v>83394</v>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Esso</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>4064 Fraser St</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.248864, 'Longitude': -123.09002}</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:12:27.452Z</t>
+        </is>
+      </c>
+      <c r="G663" t="n">
+        <v>161.9</v>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:01:42.428Z</t>
+        </is>
+      </c>
+      <c r="I663" t="n">
+        <v>197.9</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="n">
+        <v>65573</v>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>1396 E 41st Ave</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.232593005895, 'Longitude': -123.07728856802}</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>2025-08-20T03:48:05.113Z</t>
+        </is>
+      </c>
+      <c r="G664" t="n">
+        <v>160.9</v>
+      </c>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>2025-08-19T12:24:57.478Z</t>
+        </is>
+      </c>
+      <c r="I664" t="n">
+        <v>197.9</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="n">
+        <v>80714</v>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Husky</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>4933 Victoria Dr</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.2397388, 'Longitude': -123.065748}</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>2025-08-20T03:42:20.723Z</t>
+        </is>
+      </c>
+      <c r="G665" t="n">
+        <v>156.9</v>
+      </c>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:53:12.369Z</t>
+        </is>
+      </c>
+      <c r="I665" t="n">
+        <v>189.9</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="n">
+        <v>65552</v>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Esso</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>2001 Kingsway</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.245312771918, 'Longitude': -123.064910173416}</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:22:00.873Z</t>
+        </is>
+      </c>
+      <c r="G666" t="n">
+        <v>155.9</v>
+      </c>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:22:00.919Z</t>
+        </is>
+      </c>
+      <c r="I666" t="n">
+        <v>180.9</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="n">
+        <v>65538</v>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>5252 Victoria Dr</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.2372145, 'Longitude': -123.0650857}</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>2025-08-20T03:42:46.627Z</t>
+        </is>
+      </c>
+      <c r="G667" t="n">
+        <v>157.9</v>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>2025-08-20T01:06:44.322Z</t>
+        </is>
+      </c>
+      <c r="I667" t="n">
+        <v>186.9</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="n">
+        <v>90814</v>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>2277 Kingsway</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.242132845692, 'Longitude': -123.058204650879}</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:52:59.976Z</t>
+        </is>
+      </c>
+      <c r="G668" t="n">
+        <v>155.9</v>
+      </c>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:53:00.012Z</t>
+        </is>
+      </c>
+      <c r="I668" t="n">
+        <v>180.9</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="n">
+        <v>39768</v>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>5736 Main St</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.2325708, 'Longitude': -123.1010069}</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:55:11.332Z</t>
+        </is>
+      </c>
+      <c r="G669" t="n">
+        <v>156.9</v>
+      </c>
+      <c r="H669" t="inlineStr">
+        <is>
+          <t>2025-08-20T00:38:37.384Z</t>
+        </is>
+      </c>
+      <c r="I669" t="n">
+        <v>193.9</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="n">
+        <v>9710</v>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>1295 E 12th Ave</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.259878978744, 'Longitude': -123.078074455261}</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:21:28.785Z</t>
+        </is>
+      </c>
+      <c r="G670" t="n">
+        <v>156.9</v>
+      </c>
+      <c r="H670" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:21:28.848Z</t>
+        </is>
+      </c>
+      <c r="I670" t="n">
+        <v>186.9</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="n">
+        <v>99146</v>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Super Save Gas</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>1317 E 12th Ave</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.259758544957, 'Longitude': -123.077272474766}</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:21:18.799Z</t>
+        </is>
+      </c>
+      <c r="G671" t="n">
+        <v>155.9</v>
+      </c>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>2025-08-20T03:07:50.993Z</t>
+        </is>
+      </c>
+      <c r="I671" t="n">
+        <v>186.9</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="n">
+        <v>65560</v>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>1289 E Broadway</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.262693682723, 'Longitude': -123.078117370605}</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:21:17.777Z</t>
+        </is>
+      </c>
+      <c r="G672" t="n">
+        <v>155.9</v>
+      </c>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>2025-08-20T03:07:33.651Z</t>
+        </is>
+      </c>
+      <c r="I672" t="n">
+        <v>180.9</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="n">
+        <v>65557</v>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>2120 Grandview Hwy S</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.2591601, 'Longitude': -123.0617495}</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:24:44.518Z</t>
+        </is>
+      </c>
+      <c r="G673" t="n">
+        <v>157.9</v>
+      </c>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:24:48.707Z</t>
+        </is>
+      </c>
+      <c r="I673" t="n">
+        <v>183.9</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="n">
+        <v>71502</v>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>2748 Main St</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.2604441, 'Longitude': -123.1005869}</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:26:29.676Z</t>
+        </is>
+      </c>
+      <c r="G674" t="n">
+        <v>157.9</v>
+      </c>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>2025-08-19T21:21:33.123Z</t>
+        </is>
+      </c>
+      <c r="I674" t="n">
+        <v>189.9</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="n">
+        <v>65559</v>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>6502 Victoria Dr</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.224996944057, 'Longitude': -123.065521717072}</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>2025-08-20T03:49:37.095Z</t>
+        </is>
+      </c>
+      <c r="G675" t="n">
+        <v>160.9</v>
+      </c>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>2025-08-19T19:59:10.689Z</t>
+        </is>
+      </c>
+      <c r="I675" t="n">
+        <v>192.9</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="n">
+        <v>89943</v>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>6808 Victoria Dr</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.2220242, 'Longitude': -123.0654247}</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>2025-08-20T01:23:29.099Z</t>
+        </is>
+      </c>
+      <c r="G676" t="n">
+        <v>157.9</v>
+      </c>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>2025-08-19T19:59:15.108Z</t>
+        </is>
+      </c>
+      <c r="I676" t="n">
+        <v>193.9</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="n">
+        <v>86880</v>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>7282 Knight St</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.218250007984, 'Longitude': -123.076816499233}</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>2025-08-20T02:43:19.274Z</t>
+        </is>
+      </c>
+      <c r="G677" t="n">
+        <v>164.9</v>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>2025-08-19T15:14:14.480Z</t>
+        </is>
+      </c>
+      <c r="I677" t="n">
+        <v>195.9</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="n">
+        <v>65537</v>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>2918 Kingsway</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.23608, 'Longitude': -123.0454858}</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:26:21.446Z</t>
+        </is>
+      </c>
+      <c r="G678" t="n">
+        <v>157.9</v>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:26:21.493Z</t>
+        </is>
+      </c>
+      <c r="I678" t="n">
+        <v>183.9</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="n">
+        <v>65536</v>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>7309 Knight St</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.2177761, 'Longitude': -123.0775405}</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>2025-08-20T03:12:58.540Z</t>
+        </is>
+      </c>
+      <c r="G679" t="n">
+        <v>156.9</v>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>2025-08-19T15:14:04.724Z</t>
+        </is>
+      </c>
+      <c r="I679" t="n">
+        <v>193.9</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="n">
+        <v>65535</v>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>2605 E 49th Ave</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.2251291, 'Longitude': -123.0545048}</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>2025-08-20T02:00:06.584Z</t>
+        </is>
+      </c>
+      <c r="G680" t="n">
+        <v>160.9</v>
+      </c>
+      <c r="H680" t="inlineStr"/>
+      <c r="I680" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="n">
+        <v>65539</v>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>2902 Grandview Hwy</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.2579053, 'Longitude': -123.0438464}</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:40:16</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:38:57.148Z</t>
+        </is>
+      </c>
+      <c r="G681" t="n">
+        <v>157.9</v>
+      </c>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>2025-08-20T03:32:43.274Z</t>
+        </is>
+      </c>
+      <c r="I681" t="n">
+        <v>183.9</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>77015</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Super Save Gas</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>6000 No 5 Rd</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.169873456637, 'Longitude': -123.091178619746}</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:31:08.938Z</t>
+        </is>
+      </c>
+      <c r="G682" t="n">
+        <v>152.9</v>
+      </c>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:31:09.788Z</t>
+        </is>
+      </c>
+      <c r="I682" t="n">
+        <v>177.9</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>65511</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 12011 Bridgeport Rd</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.1923857, 'Longitude': -123.0911072}</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:26:17.849Z</t>
+        </is>
+      </c>
+      <c r="G683" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>2025-08-19T22:02:10.241Z</t>
+        </is>
+      </c>
+      <c r="I683" t="n">
+        <v>192.9</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>86650</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Esso</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>9100 Westminster Hwy</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.169856952787, 'Longitude': -123.123961687088}</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:43:58.858Z</t>
+        </is>
+      </c>
+      <c r="G684" t="n">
+        <v>155.9</v>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>2025-08-20T01:55:51.764Z</t>
+        </is>
+      </c>
+      <c r="I684" t="n">
+        <v>184.9</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>77218</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>5511 Garden City Rd</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.173339635958, 'Longitude': -123.124954104424}</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:05:36.665Z</t>
+        </is>
+      </c>
+      <c r="G685" t="n">
+        <v>157.9</v>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:05:36.774Z</t>
+        </is>
+      </c>
+      <c r="I685" t="n">
+        <v>187.9</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>77228</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>9100 Cambie Rd</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.1843249, 'Longitude': -123.1236078}</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>2025-08-20T03:56:31.374Z</t>
+        </is>
+      </c>
+      <c r="G686" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>2025-08-20T03:56:31.406Z</t>
+        </is>
+      </c>
+      <c r="I686" t="n">
+        <v>185.9</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>83384</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Esso</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>9060 Bridgeport Rd</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.192001, 'Longitude': -123.124004}</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:26:37.349Z</t>
+        </is>
+      </c>
+      <c r="G687" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>2025-08-19T19:33:12.509Z</t>
+        </is>
+      </c>
+      <c r="I687" t="n">
+        <v>192.9</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>77202</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>8151 Granville Ave</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.162989071149, 'Longitude': -123.134229183197}</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:33:01.855Z</t>
+        </is>
+      </c>
+      <c r="G688" t="n">
+        <v>153.9</v>
+      </c>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:56:29.411Z</t>
+        </is>
+      </c>
+      <c r="I688" t="n">
+        <v>179.9</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>77243</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Mobil</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>4651 No  3 Rd</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.179182137142, 'Longitude': -123.137152791023}</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>2025-08-20T04:36:53.942Z</t>
+        </is>
+      </c>
+      <c r="G689" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>2025-08-20T05:24:58.074Z</t>
+        </is>
+      </c>
+      <c r="I689" t="n">
+        <v>184.9</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>83387</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>710 SE Marine Dr</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.21081995506, 'Longitude': -123.090755939484}</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>2025-08-20T02:29:19.613Z</t>
+        </is>
+      </c>
+      <c r="G690" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>2025-08-20T01:30:19.967Z</t>
+        </is>
+      </c>
+      <c r="I690" t="n">
+        <v>188.9</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>65551</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Esso</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>688 SE Marine Dr</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.210798928329, 'Longitude': -123.09152841568}</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>2025-08-20T02:32:13.071Z</t>
+        </is>
+      </c>
+      <c r="G691" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>2025-08-19T14:59:32.762Z</t>
+        </is>
+      </c>
+      <c r="I691" t="n">
+        <v>192.9</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>77235</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Domo</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4071 No 3 Rd </t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>{'Latitude': None, 'Longitude': None}</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr"/>
+      <c r="G692" t="inlineStr"/>
+      <c r="H692" t="inlineStr"/>
+      <c r="I692" t="inlineStr"/>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>82925</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Mobil</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>350 SE Marine Dr</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>{'Latitude': None, 'Longitude': None}</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr"/>
+      <c r="G693" t="inlineStr"/>
+      <c r="H693" t="inlineStr"/>
+      <c r="I693" t="inlineStr"/>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>109205</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>11991 Steveston Hwy</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>{'Latitude': None, 'Longitude': None}</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr"/>
+      <c r="G694" t="inlineStr"/>
+      <c r="H694" t="inlineStr"/>
+      <c r="I694" t="inlineStr"/>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>65540</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>196 SE Marine Dr</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>{'Latitude': None, 'Longitude': None}</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr"/>
+      <c r="G695" t="inlineStr"/>
+      <c r="H695" t="inlineStr"/>
+      <c r="I695" t="inlineStr"/>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>65512</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>11131 No 5 Rd</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>{'Latitude': None, 'Longitude': None}</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr"/>
+      <c r="G696" t="inlineStr"/>
+      <c r="H696" t="inlineStr"/>
+      <c r="I696" t="inlineStr"/>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>77205</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7951 No 3 Rd </t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>{'Latitude': None, 'Longitude': None}</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr"/>
+      <c r="G697" t="inlineStr"/>
+      <c r="H697" t="inlineStr"/>
+      <c r="I697" t="inlineStr"/>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>65536</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>7309 Knight St</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>{'Latitude': None, 'Longitude': None}</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr"/>
+      <c r="G698" t="inlineStr"/>
+      <c r="H698" t="inlineStr"/>
+      <c r="I698" t="inlineStr"/>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>86880</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Petro-Canada</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>7282 Knight St</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>{'Latitude': None, 'Longitude': None}</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr"/>
+      <c r="G699" t="inlineStr"/>
+      <c r="H699" t="inlineStr"/>
+      <c r="I699" t="inlineStr"/>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>65556</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Esso</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>709 SW Marine Dr</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>{'Latitude': None, 'Longitude': None}</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr"/>
+      <c r="G700" t="inlineStr"/>
+      <c r="H700" t="inlineStr"/>
+      <c r="I700" t="inlineStr"/>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>86937</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>8655 Boundary Rd</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>{'Latitude': 49.20476, 'Longitude': -123.02398}</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>2025-08-19 22:41:32</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>2025-08-20T03:08:31.375Z</t>
+        </is>
+      </c>
+      <c r="G701" t="n">
+        <v>167.9</v>
+      </c>
+      <c r="H701" t="inlineStr">
+        <is>
+          <t>2025-08-19T16:02:16.797Z</t>
+        </is>
+      </c>
+      <c r="I701" t="n">
+        <v>197.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>